<commit_message>
Update metadata import scripts
</commit_message>
<xml_diff>
--- a/imports/templates/OmicsPred_Submission_Template.xlsx
+++ b/imports/templates/OmicsPred_Submission_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lg10/Workspace/git/fork/omicspred_backend/imports/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84E3B274-F0D2-D842-88D2-EFC43BA01374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD441DB9-2F7B-C542-A7B7-131F2387EF8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="33300" yWindow="1240" windowWidth="30240" windowHeight="17380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
   <si>
     <r>
       <rPr>
@@ -31,6 +31,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Score Name/ID
 </t>
@@ -40,6 +41,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(must be unique and consistent with the trait score filename uploaded; recommend to use the identifier provided by the assaying platform or OMICSPRED ID if existing scores for the trait are already available on OmicsPred)</t>
     </r>
@@ -57,6 +59,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Curation Notes
 </t>
@@ -66,6 +69,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(Supporting information with any details about the score that OmicsPred curators should know about</t>
     </r>
@@ -75,6 +79,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> - not displayed in the online portal</t>
     </r>
@@ -83,6 +88,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>)</t>
     </r>
@@ -94,6 +100,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Reported Trait</t>
     </r>
@@ -102,6 +109,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> 
 (omic trait that the genetic score predicts)</t>
@@ -114,6 +122,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Platform Name
 (</t>
@@ -123,6 +132,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">platform used to assay the reported trait, e.g. SomaScan, Olink. </t>
     </r>
@@ -132,6 +142,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>This refers to the trait data used in the score development stage</t>
     </r>
@@ -141,6 +152,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>)</t>
     </r>
@@ -152,6 +164,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Platform Version
 </t>
@@ -161,6 +174,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">(version of the applied platform, e.g. SomaScan version 3 - </t>
     </r>
@@ -170,6 +184,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>can ignore if not applicable</t>
     </r>
@@ -178,6 +193,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">. </t>
     </r>
@@ -187,6 +203,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>This refers to the trait data used in the score development stage</t>
     </r>
@@ -195,6 +212,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>)</t>
     </r>
@@ -206,6 +224,358 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Additional Trait Information
+(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>info that should be attached to the genetic score rather than samples, e.g. gene name, UniProt ID, pathways.  Multiple columns can be used where multiple fields of additional information are available for the omic trait</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Score Development Method
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(e.g. Elastic Net, Bayesian Ridge, LDpred, PRSice, P+T, lassosum) </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Score Development Details
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(describe key parameters used in the score development. e.g. LD/SNP r2 threshold, significance/p-value threshold, fraction of causal variants (ρ), or hyperparameters applied in machine learning methods)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Genome Build
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Original genome build the variants/genetic scores are associated with)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Number of </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>variants</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> included in genetic score
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(will be used for cross-referencing with the score file)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Number of </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>interaction terms</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> included in the genetic score
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>specify if applicable</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>; will be used for cross-referencing with the score file)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Sample Information
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(this section describes information about sets of sample collections/cohorts that correspond to different study stages (variant associations / score development / validation) of a trait. When multiple traits share the same sample set, rows of this section can be merged for these traits, e.g. the same sample set was used to validate performance of genetic scores of multiple traits)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Performance Metrics</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+(specify when applicable, e.g. performance reported at the score development stage (training sample set), performance reported at the validation stage (validation sample set))</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Associated Score Name/ID
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(must match score name/ID in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Score Information sheet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Study Stage
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Variant associations / Score development / Validation)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Platform Version
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(specify </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>ONLY</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> if this is different from the platform version used for score development, e.g. in the validation stage SomaScan v4 omics data were used to validate genetic scores developed using SomaScan v3 data)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Tissue Name
 </t>
@@ -215,25 +585,28 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">(tissue on which the assay was performed to measure the trait levels, e.g. plasma, serum, etc. </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>This refers to the trait data used in the score development stage</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>)</t>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(specify </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>ONLY</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> if this is different from the tissue on which the omics data were assayed for genetic score development, e.g. omics data for genetic scores were assayed on plasma samples but serum were used for omics data assaying in the validation)</t>
     </r>
   </si>
   <si>
@@ -243,26 +616,19 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-      </rPr>
-      <t>Additional Trait Information
-(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>info that should be attached to the genetic score rather than samples, e.g. gene name, UniProt ID, pathways.  Multiple columns can be used where multiple fields of additional information are available for the omic trait</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>)</t>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Source GWAS Catalog
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(GCST ID in the GWAS Catalog if applicable, e.g. summary stats used for variant associations and/or score development)</t>
     </r>
   </si>
   <si>
@@ -272,369 +638,26 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Score Development Method
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">(e.g. Elastic Net, Bayesian Ridge, LDpred, PRSice, P+T, lassosum) </t>
-    </r>
-  </si>
-  <si>
+        <family val="2"/>
+      </rPr>
+      <t>PMID</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> or </t>
+    </r>
     <r>
       <rPr>
         <b/>
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Score Development Details
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>(describe key parameters used in the score development. e.g. LD/SNP r2 threshold, significance/p-value threshold, fraction of causal variants (ρ), or hyperparameters applied in machine learning methods)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Genome Build
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>(Original genome build the variants/genetic scores are associated with)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Number of </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>variants</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve"> included in genetic score
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>(will be used for cross-referencing with the score file)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Number of </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>interaction terms</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve"> included in the genetic score
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>specify if applicable</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>; will be used for cross-referencing with the score file)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Sample Information
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>(this section describes information about sets of sample collections/cohorts that correspond to different study stages (variant associations / score development / validation) of a trait. When multiple traits share the same sample set, rows of this section can be merged for these traits, e.g. the same sample set was used to validate performance of genetic scores of multiple traits)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>Performance Metrics</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">
-(specify when applicable, e.g. performance reported at the score development stage (training sample set), performance reported at the validation stage (validation sample set))</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Associated Score Name/ID
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">(must match score name/ID in </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>Score Information sheet</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Study Stage
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>(Variant associations / Score development / Validation)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Platform Version
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">(specify </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>ONLY</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve"> if this is different from the platform version used for score development, e.g. in the validation stage SomaScan v4 omics data were used to validate genetic scores developed using SomaScan v3 data)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Tissue Name
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">(specify </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>ONLY</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve"> if this is different from the tissue on which the omics data were assayed for genetic score development, e.g. omics data for genetic scores were assayed on plasma samples but serum were used for omics data assaying in the validation)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Source GWAS Catalog
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>(GCST ID in the GWAS Catalog if applicable, e.g. summary stats used for variant associations and/or score development)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>PMID</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve"> or </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">DOI
 </t>
@@ -644,6 +667,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(Publication(s) that described the sample collections/cohorts used. If this is provided in the current publication, describing the genetic scores you are submitting, rather than elsewhere, just specify "current publication")</t>
     </r>
@@ -659,6 +683,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Percent of individuals who are Male
 </t>
@@ -668,6 +693,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(if known)</t>
     </r>
@@ -679,6 +705,7 @@
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Age of individuals in the collections/cohorts
 </t>
@@ -688,6 +715,7 @@
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(if known)</t>
     </r>
@@ -699,6 +727,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Broad Ancestral Category
 </t>
@@ -708,6 +737,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">(select from drop down list; more details on the listed ancestral categories can be found in table 1 of this publication </t>
     </r>
@@ -717,6 +747,7 @@
         <sz val="12"/>
         <color rgb="FF1155CC"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>https://doi.org/10.1186/s13059-018-1396-2)</t>
     </r>
@@ -728,6 +759,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Ancestry
 </t>
@@ -737,6 +769,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(e.g. French, Chinese)</t>
     </r>
@@ -748,6 +781,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Country of recruitment
 </t>
@@ -757,6 +791,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(comma separated list)</t>
     </r>
@@ -771,6 +806,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Covariates Adjustment
 </t>
@@ -780,6 +816,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(a list of covariates for which the trait levels were adjusted before the association/development/validation analyses; or a list of covariates that were included in the association/development/validation analyses, e.g. age, age2, sex, genetic PCs, batches)</t>
     </r>
@@ -791,6 +828,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Additional information on the covariates adjustment 
 </t>
@@ -800,6 +838,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">(e.g. adjustment methods used) </t>
     </r>
@@ -811,6 +850,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Cohort(s)
 </t>
@@ -820,6 +860,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">(provide a comma-separated list of Cohort IDs used in each phase, details of which should be listed in the </t>
     </r>
@@ -829,6 +870,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Cohort Information sheet</t>
     </r>
@@ -837,6 +879,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>)</t>
     </r>
@@ -848,6 +891,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Additional Sample/Cohort Information </t>
     </r>
@@ -856,6 +900,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(relevant information not captured by the structured fields)</t>
     </r>
@@ -867,6 +912,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Curation Notes
 </t>
@@ -876,6 +922,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(Supporting information with any details about the samples   -</t>
     </r>
@@ -885,6 +932,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> not displayed in the OmicsPred</t>
     </r>
@@ -893,6 +941,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>)</t>
     </r>
@@ -910,6 +959,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Additional validation performance metrics/details </t>
     </r>
@@ -918,6 +968,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(multiple columns can be applied)</t>
     </r>
@@ -927,6 +978,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -939,6 +991,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Curation Notes
 </t>
@@ -948,6 +1001,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(Supporting information with any details about the performance metric [e.g. figure/table source]  -</t>
     </r>
@@ -957,6 +1011,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> not displayed in the OmicsPred</t>
     </r>
@@ -965,6 +1020,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>)</t>
     </r>
@@ -985,6 +1041,7 @@
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Cohort </t>
     </r>
@@ -993,6 +1050,7 @@
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 (Cohort IDs used in the </t>
@@ -1003,6 +1061,7 @@
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Sample Information sheet</t>
     </r>
@@ -1011,6 +1070,7 @@
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>)</t>
     </r>
@@ -1025,6 +1085,7 @@
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>PubMed ID or doi</t>
     </r>
@@ -1033,6 +1094,7 @@
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 (publication(s) that describe the cohort and the related omic traits analyses, e.g their quality control)</t>
@@ -1045,6 +1107,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">PubMed ID
 </t>
@@ -1054,6 +1117,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(PMID)</t>
     </r>
@@ -1071,6 +1135,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Publication Date
 </t>
@@ -1080,6 +1145,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(e.g. dd-mm-yyyy)</t>
     </r>
@@ -1091,6 +1157,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>First Author Last Name</t>
     </r>
@@ -1099,6 +1166,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 </t>
@@ -1111,6 +1179,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">First Author Middle Name
 </t>
@@ -1120,6 +1189,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>(if applicable)</t>
     </r>
@@ -1139,6 +1209,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Publication Curation Notes
 </t>
@@ -1148,6 +1219,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">(Supporting information with any details about the publication that OmicsPred curators should know - </t>
     </r>
@@ -1157,6 +1229,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>not displayed in the online portal</t>
     </r>
@@ -1165,6 +1238,56 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Tissue ID
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Ontology ID corresponding to the Tissue Name)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Tissue Name
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(tissue on which the assay was performed to measure the trait levels, e.g. plasma, serum, etc. </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>This refers to the trait data used in the score development stage</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>)</t>
     </r>
@@ -1189,32 +1312,38 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1222,11 +1351,13 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1234,24 +1365,28 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="12"/>
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1690,14 +1825,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1712,23 +1857,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2017,27 +2152,29 @@
       <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="2"/>
+      <c r="E2" s="2" t="s">
+        <v>52</v>
+      </c>
       <c r="F2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>13</v>
       </c>
       <c r="M2" s="32"/>
       <c r="N2" s="1"/>
@@ -2091,8 +2228,8 @@
   <sheetData>
     <row r="1" spans="1:25" ht="101.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="6"/>
-      <c r="B1" s="37" t="s">
-        <v>14</v>
+      <c r="B1" s="41" t="s">
+        <v>13</v>
       </c>
       <c r="C1" s="29"/>
       <c r="D1" s="29"/>
@@ -2110,8 +2247,8 @@
       <c r="P1" s="29"/>
       <c r="Q1" s="29"/>
       <c r="R1" s="30"/>
-      <c r="S1" s="38" t="s">
-        <v>15</v>
+      <c r="S1" s="42" t="s">
+        <v>14</v>
       </c>
       <c r="T1" s="29"/>
       <c r="U1" s="29"/>
@@ -2121,109 +2258,109 @@
       <c r="Y1" s="7"/>
     </row>
     <row r="2" spans="1:25" ht="101.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="43" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="41" t="s">
+      <c r="C2" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="35" t="s">
+      <c r="D2" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="35" t="s">
+      <c r="E2" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="35" t="s">
+      <c r="F2" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="35" t="s">
+      <c r="G2" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="45" t="s">
+      <c r="H2" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="46" t="s">
+      <c r="I2" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="47" t="s">
+      <c r="J2" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="J2" s="48" t="s">
+      <c r="K2" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="49" t="s">
+      <c r="L2" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="L2" s="49" t="s">
+      <c r="M2" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="M2" s="47" t="s">
+      <c r="N2" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="N2" s="35" t="s">
+      <c r="O2" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="O2" s="35" t="s">
+      <c r="P2" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="P2" s="35" t="s">
+      <c r="Q2" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="Q2" s="35" t="s">
+      <c r="R2" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="R2" s="43" t="s">
+      <c r="S2" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="S2" s="33" t="s">
+      <c r="T2" s="38"/>
+      <c r="U2" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="T2" s="34"/>
-      <c r="U2" s="33" t="s">
+      <c r="V2" s="38"/>
+      <c r="W2" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="V2" s="34"/>
-      <c r="W2" s="35" t="s">
+      <c r="X2" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="X2" s="43" t="s">
+      <c r="Y2" s="7"/>
+    </row>
+    <row r="3" spans="1:25" ht="174" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="44"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="34"/>
+      <c r="J3" s="34"/>
+      <c r="K3" s="34"/>
+      <c r="L3" s="34"/>
+      <c r="M3" s="34"/>
+      <c r="N3" s="34"/>
+      <c r="O3" s="34"/>
+      <c r="P3" s="34"/>
+      <c r="Q3" s="34"/>
+      <c r="R3" s="36"/>
+      <c r="S3" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="Y2" s="7"/>
-    </row>
-    <row r="3" spans="1:25" ht="174" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="40"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
-      <c r="M3" s="36"/>
-      <c r="N3" s="36"/>
-      <c r="O3" s="36"/>
-      <c r="P3" s="36"/>
-      <c r="Q3" s="36"/>
-      <c r="R3" s="44"/>
-      <c r="S3" s="8" t="s">
+      <c r="T3" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="T3" s="8" t="s">
+      <c r="U3" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="U3" s="8" t="s">
-        <v>40</v>
+      <c r="V3" s="8" t="s">
+        <v>38</v>
       </c>
-      <c r="V3" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="W3" s="36"/>
-      <c r="X3" s="44"/>
+      <c r="W3" s="34"/>
+      <c r="X3" s="36"/>
       <c r="Y3" s="7"/>
     </row>
     <row r="4" spans="1:25" ht="13" x14ac:dyDescent="0.15">
@@ -5225,14 +5362,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="Q2:Q3"/>
-    <mergeCell ref="R2:R3"/>
-    <mergeCell ref="S2:T2"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
     <mergeCell ref="U2:V2"/>
     <mergeCell ref="W2:W3"/>
     <mergeCell ref="B1:R1"/>
@@ -5249,6 +5378,14 @@
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K3"/>
+    <mergeCell ref="Q2:Q3"/>
+    <mergeCell ref="R2:R3"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="J4:J1002" xr:uid="{00000000-0002-0000-0100-000000000000}">
@@ -5277,13 +5414,13 @@
   <sheetData>
     <row r="1" spans="1:26" ht="72.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="C1" s="12" t="s">
         <v>42</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>43</v>
       </c>
       <c r="D1" s="13"/>
       <c r="E1" s="13"/>
@@ -5332,30 +5469,30 @@
     <row r="1" spans="1:8" ht="51" x14ac:dyDescent="0.15">
       <c r="A1" s="14"/>
       <c r="B1" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="E1" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="F1" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="G1" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="H1" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="H1" s="18" t="s">
-        <v>50</v>
-      </c>
     </row>
     <row r="2" spans="1:8" ht="63.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="21"/>
@@ -5367,7 +5504,7 @@
     </row>
     <row r="3" spans="1:8" ht="102" x14ac:dyDescent="0.15">
       <c r="A3" s="25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B3" s="50"/>
       <c r="C3" s="51"/>

</xml_diff>